<commit_message>
feat: add login history permission and update related permission checks in the authentication module
</commit_message>
<xml_diff>
--- a/postcheck.xlsx
+++ b/postcheck.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srivatsan/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srivatsan/Desktop/ai-consulting-platform/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C2DB43-34AD-EF44-9230-8E528D107EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F661FB9-6385-8345-B6FB-8CB5014672CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="16640" activeTab="4" xr2:uid="{706BB7B9-90F1-D04B-AFED-02F89A0AB2A0}"/>
+    <workbookView minimized="1" xWindow="0" yWindow="940" windowWidth="30240" windowHeight="16640" activeTab="2" xr2:uid="{706BB7B9-90F1-D04B-AFED-02F89A0AB2A0}"/>
   </bookViews>
   <sheets>
     <sheet name="saas(missing)" sheetId="2" r:id="rId1"/>

</xml_diff>